<commit_message>
test: controlar ejecucion y datos desde Excel
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -2,7 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="login" sheetId="1" r:id="Rec366aff845d4aa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="login" sheetId="1" r:id="Rc94c9f0395d64974"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="execution" sheetId="2" r:id="R631faf3f9e304b13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="employee" sheetId="3" r:id="R06ac13c7d246410a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -39,7 +41,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -56,6 +58,11 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -63,7 +70,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -98,12 +105,100 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ExecutionTable" displayName="ExecutionTable" ref="A1:F6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="caseId"/>
+    <x:tableColumn id="2" name="enabled"/>
+    <x:tableColumn id="3" name="chrome"/>
+    <x:tableColumn id="4" name="firefox"/>
+    <x:tableColumn id="5" name="edge"/>
+    <x:tableColumn id="6" name="dataSheet"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EmployeeDataTable" displayName="EmployeeDataTable" ref="A1:I4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="caseId"/>
+    <x:tableColumn id="2" name="dataId"/>
+    <x:tableColumn id="3" name="firstNameMode"/>
+    <x:tableColumn id="4" name="firstNamePrefix"/>
+    <x:tableColumn id="5" name="middleName"/>
+    <x:tableColumn id="6" name="lastNamePrefix"/>
+    <x:tableColumn id="7" name="searchBy"/>
+    <x:tableColumn id="8" name="expectedResult"/>
+    <x:tableColumn id="9" name="expectedMessage"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -375,4 +470,280 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="19" t="str">
+        <x:v>caseId</x:v>
+      </x:c>
+      <x:c r="B1" s="19" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="C1" s="19" t="str">
+        <x:v>chrome</x:v>
+      </x:c>
+      <x:c r="D1" s="19" t="str">
+        <x:v>firefox</x:v>
+      </x:c>
+      <x:c r="E1" s="19" t="str">
+        <x:v>edge</x:v>
+      </x:c>
+      <x:c r="F1" s="19" t="str">
+        <x:v>dataSheet</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="20" t="str">
+        <x:v>TC01</x:v>
+      </x:c>
+      <x:c r="B2" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="C2" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="D2" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="E2" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="F2" s="20" t="str">
+        <x:v>login</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="20" t="str">
+        <x:v>TC02</x:v>
+      </x:c>
+      <x:c r="B3" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="C3" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="D3" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="E3" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="F3" s="20" t="str">
+        <x:v>login</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="20" t="str">
+        <x:v>TC06</x:v>
+      </x:c>
+      <x:c r="B4" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="C4" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="D4" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="E4" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="F4" s="20" t="str">
+        <x:v>employee</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="20" t="str">
+        <x:v>TC07</x:v>
+      </x:c>
+      <x:c r="B5" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="C5" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="D5" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="E5" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="F5" s="20" t="str">
+        <x:v>employee</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="20" t="str">
+        <x:v>TC08</x:v>
+      </x:c>
+      <x:c r="B6" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="C6" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="D6" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="E6" s="20" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="F6" s="20" t="str">
+        <x:v>employee</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="B2:E6">
+      <x:formula1>"TRUE,FALSE"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdeb22b265fa54dfa"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="24" t="str">
+        <x:v>caseId</x:v>
+      </x:c>
+      <x:c r="B1" s="24" t="str">
+        <x:v>dataId</x:v>
+      </x:c>
+      <x:c r="C1" s="24" t="str">
+        <x:v>firstNameMode</x:v>
+      </x:c>
+      <x:c r="D1" s="24" t="str">
+        <x:v>firstNamePrefix</x:v>
+      </x:c>
+      <x:c r="E1" s="24" t="str">
+        <x:v>middleName</x:v>
+      </x:c>
+      <x:c r="F1" s="24" t="str">
+        <x:v>lastNamePrefix</x:v>
+      </x:c>
+      <x:c r="G1" s="24" t="str">
+        <x:v>searchBy</x:v>
+      </x:c>
+      <x:c r="H1" s="24" t="str">
+        <x:v>expectedResult</x:v>
+      </x:c>
+      <x:c r="I1" s="24" t="str">
+        <x:v>expectedMessage</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="20" t="str">
+        <x:v>TC06</x:v>
+      </x:c>
+      <x:c r="B2" s="20" t="str">
+        <x:v>EMPLOYEE_VALID</x:v>
+      </x:c>
+      <x:c r="C2" s="20" t="str">
+        <x:v>AUTO</x:v>
+      </x:c>
+      <x:c r="D2" s="20" t="str">
+        <x:v>Auto</x:v>
+      </x:c>
+      <x:c r="E2" s="20" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="F2" s="20" t="str">
+        <x:v>TC06</x:v>
+      </x:c>
+      <x:c r="G2" s="20" t="str"/>
+      <x:c r="H2" s="20" t="str">
+        <x:v>success</x:v>
+      </x:c>
+      <x:c r="I2" s="20" t="str">
+        <x:v>Personal Details</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="20" t="str">
+        <x:v>TC07</x:v>
+      </x:c>
+      <x:c r="B3" s="20" t="str">
+        <x:v>EMPLOYEE_SEARCH</x:v>
+      </x:c>
+      <x:c r="C3" s="20" t="str">
+        <x:v>AUTO</x:v>
+      </x:c>
+      <x:c r="D3" s="20" t="str">
+        <x:v>Auto</x:v>
+      </x:c>
+      <x:c r="E3" s="20" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="F3" s="20" t="str">
+        <x:v>TC07</x:v>
+      </x:c>
+      <x:c r="G3" s="20" t="str">
+        <x:v>employeeId</x:v>
+      </x:c>
+      <x:c r="H3" s="20" t="str">
+        <x:v>success</x:v>
+      </x:c>
+      <x:c r="I3" s="20" t="str">
+        <x:v>(1) Record Found</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="20" t="str">
+        <x:v>TC08</x:v>
+      </x:c>
+      <x:c r="B4" s="20" t="str">
+        <x:v>FIRST_NAME_REQUIRED</x:v>
+      </x:c>
+      <x:c r="C4" s="20" t="str">
+        <x:v>BLANK</x:v>
+      </x:c>
+      <x:c r="D4" s="20" t="str"/>
+      <x:c r="E4" s="20" t="str"/>
+      <x:c r="F4" s="20" t="str">
+        <x:v>TC08</x:v>
+      </x:c>
+      <x:c r="G4" s="20" t="str"/>
+      <x:c r="H4" s="20" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="I4" s="20" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b0145c026984e8b"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>